<commit_message>
feat(report): add rif resistance template
- add report

[Finishes ASP-1286]
</commit_message>
<xml_diff>
--- a/api/templates/rif_resistance_rate/en.xlsx
+++ b/api/templates/rif_resistance_rate/en.xlsx
@@ -1,20 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\systemoneid\aspect\api\placeholders\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6470" tabRatio="815"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6465" tabRatio="815"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="6" r:id="rId1"/>
+    <sheet name="Rif Resistance Report" sheetId="6" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" fullPrecision="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="144525" fullPrecision="0" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" Flags="2"/>
@@ -24,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Total Tests</t>
   </si>
@@ -41,88 +36,49 @@
     <t>RIF Resistance Rate</t>
   </si>
   <si>
-    <t>Date Range: 9/1/2017 - 9/28/2019</t>
-  </si>
-  <si>
     <t>State</t>
   </si>
   <si>
     <t>County</t>
   </si>
   <si>
-    <t>Shelburne Falls ML</t>
-  </si>
-  <si>
-    <t>Massachusetts</t>
-  </si>
-  <si>
-    <t>Hampshire County</t>
-  </si>
-  <si>
-    <t>Akron ML</t>
-  </si>
-  <si>
-    <t>Ohio</t>
-  </si>
-  <si>
-    <t>Summit County</t>
-  </si>
-  <si>
-    <t>Boston Micro</t>
-  </si>
-  <si>
-    <t>Suffolk County</t>
-  </si>
-  <si>
-    <t>Philadelphia ML</t>
-  </si>
-  <si>
-    <t>Pennsylvania</t>
-  </si>
-  <si>
-    <t>Philadelphia County</t>
-  </si>
-  <si>
-    <t>Pittsburgh ML</t>
-  </si>
-  <si>
-    <t>Allegheny County</t>
-  </si>
-  <si>
-    <t>Northampton ML</t>
-  </si>
-  <si>
-    <t>Wooster ML</t>
-  </si>
-  <si>
-    <t>Wayne County</t>
-  </si>
-  <si>
-    <t>Atlanta ML</t>
-  </si>
-  <si>
-    <t>Georgia</t>
-  </si>
-  <si>
-    <t>Fulton County</t>
-  </si>
-  <si>
-    <t>Cleveland ML</t>
-  </si>
-  <si>
-    <t>Cuyahoga County</t>
-  </si>
-  <si>
-    <t>Wooster Hospital</t>
-  </si>
-  <si>
     <t>Devices</t>
+  </si>
+  <si>
+    <t>Date Range: &lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>States: &lt;States&gt;</t>
+  </si>
+  <si>
+    <t>LGA: &lt;Lgas&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Table&gt;</t>
+  </si>
+  <si>
+    <t>&lt;name&gt;</t>
+  </si>
+  <si>
+    <t>&lt;state&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalResults&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalResult1&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalResult2&gt;</t>
+  </si>
+  <si>
+    <t>&lt;rifResistance&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -273,7 +229,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -289,138 +245,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -758,287 +630,93 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="27.08203125" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="3" customWidth="1"/>
-    <col min="5" max="6" width="14.83203125" customWidth="1"/>
+    <col min="1" max="3" width="27.125" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="3" customWidth="1"/>
+    <col min="5" max="6" width="14.875" customWidth="1"/>
     <col min="7" max="7" width="17.75" customWidth="1"/>
-    <col min="8" max="8" width="13.33203125" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="13.375" customWidth="1"/>
+    <col min="9" max="9" width="14.375" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="38" t="s">
+    <row r="7" spans="1:7" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="E7" s="38" t="s">
+      <c r="E7" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="F7" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="38" t="s">
+      <c r="G7" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="6">
-        <v>1927</v>
-      </c>
-      <c r="E8" s="5">
-        <v>200</v>
-      </c>
-      <c r="F8" s="5">
-        <v>164</v>
-      </c>
-      <c r="G8" s="37">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="9">
-        <v>45</v>
-      </c>
-      <c r="E9" s="10">
-        <v>9</v>
-      </c>
-      <c r="F9" s="11">
-        <v>7</v>
-      </c>
-      <c r="G9" s="37">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="33" t="s">
+      <c r="D8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="33" t="s">
+      <c r="E8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="12">
-        <v>1011</v>
-      </c>
-      <c r="E10" s="13">
-        <v>123</v>
-      </c>
-      <c r="F10" s="14">
-        <v>100</v>
-      </c>
-      <c r="G10" s="37">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="33" t="s">
+      <c r="F8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="G8" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="C11" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="15">
-        <v>24</v>
-      </c>
-      <c r="E11" s="16">
-        <v>11</v>
-      </c>
-      <c r="F11" s="17">
-        <v>9</v>
-      </c>
-      <c r="G11" s="37">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="18">
-        <v>2130</v>
-      </c>
-      <c r="E12" s="19">
-        <v>309</v>
-      </c>
-      <c r="F12" s="20">
-        <v>274</v>
-      </c>
-      <c r="G12" s="37">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="21">
-        <v>2063</v>
-      </c>
-      <c r="E13" s="22">
-        <v>348</v>
-      </c>
-      <c r="F13" s="23">
-        <v>319</v>
-      </c>
-      <c r="G13" s="37">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="24">
-        <v>2653</v>
-      </c>
-      <c r="E14" s="25">
-        <v>329</v>
-      </c>
-      <c r="F14" s="26">
-        <v>295</v>
-      </c>
-      <c r="G14" s="37">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="27">
-        <v>5</v>
-      </c>
-      <c r="E15" s="28">
-        <v>1</v>
-      </c>
-      <c r="F15" s="29">
-        <v>1</v>
-      </c>
-      <c r="G15" s="37">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="30">
-        <v>4</v>
-      </c>
-      <c r="E16" s="31">
-        <v>2</v>
-      </c>
-      <c r="F16" s="32">
-        <v>2</v>
-      </c>
-      <c r="G16" s="37">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="33" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="34">
-        <v>44</v>
-      </c>
-      <c r="E17" s="35">
-        <v>30</v>
-      </c>
-      <c r="F17" s="36">
-        <v>30</v>
-      </c>
-      <c r="G17" s="37">
-        <v>0.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(rifresistance): format excel template
</commit_message>
<xml_diff>
--- a/api/templates/rif_resistance_rate/en.xlsx
+++ b/api/templates/rif_resistance_rate/en.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\rif_resistance_rate\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="5625" yWindow="3825" windowWidth="20730" windowHeight="11145" tabRatio="815"/>
   </bookViews>
@@ -14,7 +19,7 @@
     <definedName name="totalDetected2" localSheetId="0">'Rif Resistance Report'!$G$8</definedName>
     <definedName name="totalDetected2">'Rif Resistance Report'!$F$8</definedName>
   </definedNames>
-  <calcPr calcId="144525" fullPrecision="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="144525" fullPrecision="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -94,7 +99,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -253,7 +258,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -266,17 +271,27 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="43" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="43" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="2" borderId="3" xfId="43" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="3" xfId="43" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
@@ -666,10 +681,10 @@
     <col min="1" max="1" width="39.125" customWidth="1"/>
     <col min="2" max="2" width="29.125" customWidth="1"/>
     <col min="3" max="3" width="27.125" customWidth="1"/>
-    <col min="4" max="4" width="15.375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="19.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19" style="5" customWidth="1"/>
+    <col min="4" max="4" width="12.875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.5" style="3" customWidth="1"/>
+    <col min="7" max="7" width="15.625" style="5" customWidth="1"/>
     <col min="8" max="8" width="13.375" customWidth="1"/>
     <col min="9" max="9" width="14.375" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
@@ -705,17 +720,17 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="1:7" s="11" customFormat="1" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
+    <row r="7" spans="1:7" s="8" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="11" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="9" t="s">
@@ -724,7 +739,7 @@
       <c r="F7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="13" t="s">
         <v>4</v>
       </c>
     </row>
@@ -738,16 +753,16 @@
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="6" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
- separate file for  Malawi to show County - another solution with placeholders
</commit_message>
<xml_diff>
--- a/api/templates/rif_resistance_rate/en.xlsx
+++ b/api/templates/rif_resistance_rate/en.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\rif_resistance_rate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\rif_resistance_rate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF5C8CE-AF96-4FE5-ACA2-F9844A4CADAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Rif Resistance Report" sheetId="6" r:id="rId1"/>
@@ -38,12 +37,6 @@
     <t>RIF Resistance Report</t>
   </si>
   <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>County</t>
-  </si>
-  <si>
     <t>Devices</t>
   </si>
   <si>
@@ -87,12 +80,18 @@
   </si>
   <si>
     <t>Rif Resistance Rate</t>
+  </si>
+  <si>
+    <t>&lt;CountyLabel&gt;</t>
+  </si>
+  <si>
+    <t>&lt;StateLabel&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -333,8 +332,36 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="43" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -667,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -692,22 +719,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -715,48 +742,48 @@
     </row>
     <row r="7" spans="1:7" s="8" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>16</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="F8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="10" t="s">
+      <c r="G8" s="6" t="s">
         <v>13</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>